<commit_message>
Rerun: H2-delay and fuel-availability studies on the corrected model
Licensed AMPL + Gurobi via the study drivers, S-curve demand (680 Mt),
monotonic enforced. Fuel availability: with scarce coking coal only an
H2 start in 2030 is feasible (paper: up to 2035); with abundant coal,
up to 2035 (paper: 2045 for abundant NG).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVt5c2AiN5SahjfAqCCvTJ
</commit_message>
<xml_diff>
--- a/structural/fuel_availability/data/fuel_availability.xlsx
+++ b/structural/fuel_availability/data/fuel_availability.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="17">
   <si>
     <t>Regime</t>
   </si>
@@ -71,16 +71,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -96,7 +88,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -104,30 +96,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,34 +400,34 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -471,22 +445,22 @@
         <v>2030</v>
       </c>
       <c r="E2">
-        <v>0.1992</v>
+        <v>0.3669</v>
       </c>
       <c r="F2">
-        <v>0.0818</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>0.1623</v>
+        <v>0.0854</v>
       </c>
       <c r="H2">
-        <v>0.2866</v>
+        <v>0.3315</v>
       </c>
       <c r="I2">
-        <v>0.2701</v>
+        <v>0.2161</v>
       </c>
       <c r="J2">
-        <v>388</v>
+        <v>482.3</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -503,22 +477,22 @@
         <v>2035</v>
       </c>
       <c r="E3">
-        <v>0.2568</v>
+        <v>0.4055</v>
       </c>
       <c r="F3">
-        <v>0.0558</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0.1623</v>
+        <v>0.0854</v>
       </c>
       <c r="H3">
-        <v>0.2579</v>
+        <v>0.3152</v>
       </c>
       <c r="I3">
-        <v>0.2673</v>
+        <v>0.1938</v>
       </c>
       <c r="J3">
-        <v>448.8</v>
+        <v>531.2</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -534,23 +508,23 @@
       <c r="D4">
         <v>2040</v>
       </c>
-      <c r="E4">
-        <v>0.4087</v>
-      </c>
-      <c r="F4">
-        <v>0.0115</v>
-      </c>
-      <c r="G4">
-        <v>0.1623</v>
-      </c>
-      <c r="H4">
-        <v>0.1601</v>
-      </c>
-      <c r="I4">
-        <v>0.2573</v>
-      </c>
-      <c r="J4">
-        <v>577.2</v>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -566,23 +540,23 @@
       <c r="D5">
         <v>2045</v>
       </c>
-      <c r="E5">
-        <v>0.5306999999999999</v>
-      </c>
-      <c r="F5">
-        <v>0.0177</v>
-      </c>
-      <c r="G5">
-        <v>0.1623</v>
-      </c>
-      <c r="H5">
-        <v>0.0397</v>
-      </c>
-      <c r="I5">
-        <v>0.2496</v>
-      </c>
-      <c r="J5">
-        <v>699.2</v>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -599,22 +573,22 @@
         <v>2030</v>
       </c>
       <c r="E6">
-        <v>0.2377</v>
+        <v>0.3941</v>
       </c>
       <c r="F6">
-        <v>0.1186</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>0.0537</v>
+        <v>0.0283</v>
       </c>
       <c r="H6">
-        <v>0.3217</v>
+        <v>0.3555</v>
       </c>
       <c r="I6">
-        <v>0.2682</v>
+        <v>0.2221</v>
       </c>
       <c r="J6">
-        <v>318.3</v>
+        <v>453.6</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -631,22 +605,22 @@
         <v>2035</v>
       </c>
       <c r="E7">
-        <v>0.3235</v>
+        <v>0.4809</v>
       </c>
       <c r="F7">
-        <v>0.07580000000000001</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>0.0537</v>
+        <v>0.0283</v>
       </c>
       <c r="H7">
-        <v>0.2831</v>
+        <v>0.3152</v>
       </c>
       <c r="I7">
-        <v>0.2639</v>
+        <v>0.1756</v>
       </c>
       <c r="J7">
-        <v>425.4</v>
+        <v>558.5</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -662,23 +636,23 @@
       <c r="D8">
         <v>2040</v>
       </c>
-      <c r="E8">
-        <v>0.5131</v>
-      </c>
-      <c r="F8">
-        <v>0.0214</v>
-      </c>
-      <c r="G8">
-        <v>0.0537</v>
-      </c>
-      <c r="H8">
-        <v>0.1622</v>
-      </c>
-      <c r="I8">
-        <v>0.2496</v>
-      </c>
-      <c r="J8">
-        <v>596.2</v>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -727,22 +701,22 @@
         <v>2030</v>
       </c>
       <c r="E10">
-        <v>0.1992</v>
+        <v>0.2454</v>
       </c>
       <c r="F10">
-        <v>0.0818</v>
+        <v>0.0682</v>
       </c>
       <c r="G10">
-        <v>0.1623</v>
+        <v>0.0854</v>
       </c>
       <c r="H10">
-        <v>0.2866</v>
+        <v>0.3766</v>
       </c>
       <c r="I10">
-        <v>0.2701</v>
+        <v>0.2243</v>
       </c>
       <c r="J10">
-        <v>388</v>
+        <v>338.7</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -758,23 +732,23 @@
       <c r="D11">
         <v>2035</v>
       </c>
-      <c r="E11">
-        <v>0.212</v>
-      </c>
-      <c r="F11">
-        <v>0.0926</v>
-      </c>
-      <c r="G11">
-        <v>0.1623</v>
-      </c>
-      <c r="H11">
-        <v>0.2637</v>
-      </c>
-      <c r="I11">
-        <v>0.2695</v>
-      </c>
-      <c r="J11">
-        <v>405.8</v>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -855,22 +829,22 @@
         <v>2030</v>
       </c>
       <c r="E14">
-        <v>0.212</v>
+        <v>0.2622</v>
       </c>
       <c r="F14">
-        <v>0.1391</v>
+        <v>0.0858</v>
       </c>
       <c r="G14">
-        <v>0.0537</v>
+        <v>0.0283</v>
       </c>
       <c r="H14">
-        <v>0.3257</v>
+        <v>0.4064</v>
       </c>
       <c r="I14">
-        <v>0.2695</v>
+        <v>0.2174</v>
       </c>
       <c r="J14">
-        <v>303.2</v>
+        <v>296.6</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -886,23 +860,23 @@
       <c r="D15">
         <v>2035</v>
       </c>
-      <c r="E15">
-        <v>0.2392</v>
-      </c>
-      <c r="F15">
-        <v>0.1306</v>
-      </c>
-      <c r="G15">
-        <v>0.0537</v>
-      </c>
-      <c r="H15">
-        <v>0.3083</v>
-      </c>
-      <c r="I15">
-        <v>0.2681</v>
-      </c>
-      <c r="J15">
-        <v>320.4</v>
+      <c r="E15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:10">

</xml_diff>